<commit_message>
fix: wind data has changed
</commit_message>
<xml_diff>
--- a/data/Fissures/Fissure_2.xlsx
+++ b/data/Fissures/Fissure_2.xlsx
@@ -230,7 +230,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr defaultColWidth="10.921875" defaultRowHeight="14.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.13"/>
@@ -1066,6 +1066,44 @@
         <v>-0.569999999999993</v>
       </c>
     </row>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="5" t="n">
+        <v>45564</v>
+      </c>
+      <c r="B45" s="1" t="n">
+        <v>30.08</v>
+      </c>
+      <c r="C45" s="1" t="n">
+        <v>90.73</v>
+      </c>
+      <c r="D45" s="1" t="n">
+        <f aca="false">B45-B44</f>
+        <v>0.0399999999999991</v>
+      </c>
+      <c r="E45" s="1" t="n">
+        <f aca="false">C45-C44</f>
+        <v>0.920000000000002</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="5" t="n">
+        <v>45571</v>
+      </c>
+      <c r="B46" s="1" t="n">
+        <v>30.08</v>
+      </c>
+      <c r="C46" s="1" t="n">
+        <v>90.45</v>
+      </c>
+      <c r="D46" s="1" t="n">
+        <f aca="false">B46-B45</f>
+        <v>0</v>
+      </c>
+      <c r="E46" s="1" t="n">
+        <f aca="false">C46-C45</f>
+        <v>-0.280000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>

<commit_message>
feat: add phase to LOESS
</commit_message>
<xml_diff>
--- a/data/Fissures/Fissure_2.xlsx
+++ b/data/Fissures/Fissure_2.xlsx
@@ -230,7 +230,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr defaultColWidth="10.921875" defaultRowHeight="14.5" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12.13"/>
@@ -1104,6 +1104,25 @@
         <v>-0.280000000000001</v>
       </c>
     </row>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="5" t="n">
+        <v>45578</v>
+      </c>
+      <c r="B47" s="1" t="n">
+        <v>30.02</v>
+      </c>
+      <c r="C47" s="1" t="n">
+        <v>90.69</v>
+      </c>
+      <c r="D47" s="1" t="n">
+        <f aca="false">B47-B46</f>
+        <v>-0.0599999999999987</v>
+      </c>
+      <c r="E47" s="1" t="n">
+        <f aca="false">C47-C46</f>
+        <v>0.239999999999995</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>

<commit_message>
feat: add PELT & HMM
</commit_message>
<xml_diff>
--- a/data/Fissures/Fissure_2.xlsx
+++ b/data/Fissures/Fissure_2.xlsx
@@ -108,7 +108,7 @@
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -144,13 +144,6 @@
       <name val="Calibri"/>
       <family val="1"/>
       <charset val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFC9211E"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -220,7 +213,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -233,66 +226,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FFC9211E"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -1202,7 +1135,7 @@
         <v>30.04</v>
       </c>
       <c r="C48" s="6" t="n">
-        <v>90.69</v>
+        <v>90.25</v>
       </c>
       <c r="D48" s="1" t="n">
         <f aca="false">B48-B47</f>
@@ -1210,7 +1143,7 @@
       </c>
       <c r="E48" s="1" t="n">
         <f aca="false">C48-C47</f>
-        <v>0</v>
+        <v>-0.439999999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: route + models
</commit_message>
<xml_diff>
--- a/data/Fissures/Fissure_2.xlsx
+++ b/data/Fissures/Fissure_2.xlsx
@@ -1,33 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\johan\PycharmProjects\Fissure-master\data\Fissures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4258E3BC-97BD-4BCC-B504-B8397D0A91AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4217969A-B115-4B40-8ADD-7D8025899A0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1520" yWindow="1520" windowWidth="28800" windowHeight="15910" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21820" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -36,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Date</t>
   </si>
@@ -113,6 +102,10 @@
       </rPr>
       <t>(mm)</t>
     </r>
+  </si>
+  <si>
+    <t>Mur route
+(inch)</t>
   </si>
 </sst>
 </file>
@@ -518,7 +511,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AMJ62"/>
+  <dimension ref="A1:AMJ63"/>
   <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="12.08984375" style="3" customWidth="1"/>
@@ -545,7 +538,9 @@
       <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2"/>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3">
@@ -1697,6 +1692,28 @@
       <c r="E62" s="8">
         <f t="shared" si="9"/>
         <v>-0.10000000000000853</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6">
+      <c r="A63" s="3">
+        <v>45697</v>
+      </c>
+      <c r="B63" s="6">
+        <v>30.05</v>
+      </c>
+      <c r="C63" s="6">
+        <v>91.36</v>
+      </c>
+      <c r="D63" s="8">
+        <f t="shared" ref="D63" si="10">B63-B62</f>
+        <v>0</v>
+      </c>
+      <c r="E63" s="8">
+        <f t="shared" ref="E63" si="11">C63-C62</f>
+        <v>0.12000000000000455</v>
+      </c>
+      <c r="F63" s="1">
+        <v>0.76300000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update files (with data_route)
</commit_message>
<xml_diff>
--- a/data/Fissures/Fissure_2.xlsx
+++ b/data/Fissures/Fissure_2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\johan\PycharmProjects\Fissure-master\data\Fissures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4217969A-B115-4B40-8ADD-7D8025899A0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B8E6022-DF9F-4C50-AC98-8FE64D67E91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21820" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-32070" yWindow="1620" windowWidth="16440" windowHeight="29040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -511,7 +511,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AMJ63"/>
+  <dimension ref="A1:AMJ79"/>
   <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="12.08984375" style="3" customWidth="1"/>
@@ -1712,8 +1712,309 @@
         <f t="shared" ref="E63" si="11">C63-C62</f>
         <v>0.12000000000000455</v>
       </c>
-      <c r="F63" s="1">
-        <v>0.76300000000000001</v>
+    </row>
+    <row r="64" spans="1:6">
+      <c r="A64" s="3">
+        <v>45704</v>
+      </c>
+      <c r="B64" s="6">
+        <v>30.07</v>
+      </c>
+      <c r="C64" s="6">
+        <v>91.18</v>
+      </c>
+      <c r="D64" s="8">
+        <f t="shared" ref="D64:D68" si="12">B64-B63</f>
+        <v>1.9999999999999574E-2</v>
+      </c>
+      <c r="E64" s="8">
+        <f t="shared" ref="E64:E68" si="13">C64-C63</f>
+        <v>-0.17999999999999261</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5">
+      <c r="A65" s="3">
+        <v>45711</v>
+      </c>
+      <c r="B65" s="6">
+        <v>30.1</v>
+      </c>
+      <c r="C65" s="6">
+        <v>90.7</v>
+      </c>
+      <c r="D65" s="8">
+        <f t="shared" si="12"/>
+        <v>3.0000000000001137E-2</v>
+      </c>
+      <c r="E65" s="8">
+        <f t="shared" si="13"/>
+        <v>-0.48000000000000398</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
+      <c r="A66" s="3">
+        <v>45718</v>
+      </c>
+      <c r="B66" s="6">
+        <v>30.14</v>
+      </c>
+      <c r="C66" s="6">
+        <v>90.78</v>
+      </c>
+      <c r="D66" s="8">
+        <f t="shared" si="12"/>
+        <v>3.9999999999999147E-2</v>
+      </c>
+      <c r="E66" s="8">
+        <f t="shared" si="13"/>
+        <v>7.9999999999998295E-2</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
+      <c r="A67" s="3">
+        <v>45725</v>
+      </c>
+      <c r="B67" s="6">
+        <v>30.13</v>
+      </c>
+      <c r="C67" s="6">
+        <v>90.01</v>
+      </c>
+      <c r="D67" s="8">
+        <f t="shared" si="12"/>
+        <v>-1.0000000000001563E-2</v>
+      </c>
+      <c r="E67" s="8">
+        <f t="shared" si="13"/>
+        <v>-0.76999999999999602</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
+      <c r="A68" s="3">
+        <v>45732</v>
+      </c>
+      <c r="B68" s="6">
+        <v>30.1</v>
+      </c>
+      <c r="C68" s="6">
+        <v>90.66</v>
+      </c>
+      <c r="D68" s="8">
+        <f t="shared" si="12"/>
+        <v>-2.9999999999997584E-2</v>
+      </c>
+      <c r="E68" s="8">
+        <f t="shared" si="13"/>
+        <v>0.64999999999999147</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
+      <c r="A69" s="3">
+        <v>45739</v>
+      </c>
+      <c r="B69" s="6">
+        <v>30.14</v>
+      </c>
+      <c r="C69" s="6">
+        <v>90.41</v>
+      </c>
+      <c r="D69" s="8">
+        <f t="shared" ref="D69:D70" si="14">B69-B68</f>
+        <v>3.9999999999999147E-2</v>
+      </c>
+      <c r="E69" s="8">
+        <f t="shared" ref="E69:E70" si="15">C69-C68</f>
+        <v>-0.25</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70" s="3">
+        <v>45746</v>
+      </c>
+      <c r="B70" s="6">
+        <v>30.14</v>
+      </c>
+      <c r="C70" s="6">
+        <v>90.57</v>
+      </c>
+      <c r="D70" s="8">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+      <c r="E70" s="8">
+        <f t="shared" si="15"/>
+        <v>0.15999999999999659</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71" s="3">
+        <v>45753</v>
+      </c>
+      <c r="B71" s="6">
+        <v>30.15</v>
+      </c>
+      <c r="C71" s="6">
+        <v>89.93</v>
+      </c>
+      <c r="D71" s="8">
+        <f t="shared" ref="D71:D76" si="16">B71-B70</f>
+        <v>9.9999999999980105E-3</v>
+      </c>
+      <c r="E71" s="8">
+        <f t="shared" ref="E71:E76" si="17">C71-C70</f>
+        <v>-0.63999999999998636</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5">
+      <c r="A72" s="3">
+        <v>45760</v>
+      </c>
+      <c r="B72" s="6">
+        <v>30.16</v>
+      </c>
+      <c r="C72" s="6">
+        <v>90.17</v>
+      </c>
+      <c r="D72" s="8">
+        <f t="shared" si="16"/>
+        <v>1.0000000000001563E-2</v>
+      </c>
+      <c r="E72" s="8">
+        <f t="shared" si="17"/>
+        <v>0.23999999999999488</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5">
+      <c r="A73" s="3">
+        <v>45767</v>
+      </c>
+      <c r="B73" s="6">
+        <v>30.14</v>
+      </c>
+      <c r="C73" s="6">
+        <v>90.27</v>
+      </c>
+      <c r="D73" s="8">
+        <f t="shared" si="16"/>
+        <v>-1.9999999999999574E-2</v>
+      </c>
+      <c r="E73" s="8">
+        <f t="shared" si="17"/>
+        <v>9.9999999999994316E-2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
+      <c r="A74" s="3">
+        <v>45774</v>
+      </c>
+      <c r="B74" s="6">
+        <v>30.16</v>
+      </c>
+      <c r="C74" s="6">
+        <v>90.38</v>
+      </c>
+      <c r="D74" s="8">
+        <f t="shared" si="16"/>
+        <v>1.9999999999999574E-2</v>
+      </c>
+      <c r="E74" s="8">
+        <f t="shared" si="17"/>
+        <v>0.10999999999999943</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
+      <c r="A75" s="3">
+        <v>45781</v>
+      </c>
+      <c r="B75" s="6">
+        <v>30.16</v>
+      </c>
+      <c r="C75" s="6">
+        <v>90.18</v>
+      </c>
+      <c r="D75" s="8">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="E75" s="8">
+        <f t="shared" si="17"/>
+        <v>-0.19999999999998863</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5">
+      <c r="A76" s="3">
+        <v>45788</v>
+      </c>
+      <c r="B76" s="6">
+        <v>30.17</v>
+      </c>
+      <c r="C76" s="6">
+        <v>89.89</v>
+      </c>
+      <c r="D76" s="8">
+        <f t="shared" si="16"/>
+        <v>1.0000000000001563E-2</v>
+      </c>
+      <c r="E76" s="8">
+        <f t="shared" si="17"/>
+        <v>-0.29000000000000625</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5">
+      <c r="A77" s="3">
+        <v>45795</v>
+      </c>
+      <c r="B77" s="6">
+        <v>30.2</v>
+      </c>
+      <c r="C77" s="6">
+        <v>90.42</v>
+      </c>
+      <c r="D77" s="8">
+        <f t="shared" ref="D77:D79" si="18">B77-B76</f>
+        <v>2.9999999999997584E-2</v>
+      </c>
+      <c r="E77" s="8">
+        <f t="shared" ref="E77:E79" si="19">C77-C76</f>
+        <v>0.53000000000000114</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5">
+      <c r="A78" s="3">
+        <v>45802</v>
+      </c>
+      <c r="B78" s="6">
+        <v>30.2</v>
+      </c>
+      <c r="C78" s="6">
+        <v>90.2</v>
+      </c>
+      <c r="D78" s="8">
+        <f t="shared" si="18"/>
+        <v>0</v>
+      </c>
+      <c r="E78" s="8">
+        <f t="shared" si="19"/>
+        <v>-0.21999999999999886</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5">
+      <c r="A79" s="3">
+        <v>45809</v>
+      </c>
+      <c r="B79" s="6">
+        <v>30.18</v>
+      </c>
+      <c r="C79" s="6">
+        <v>90.06</v>
+      </c>
+      <c r="D79" s="8">
+        <f t="shared" si="18"/>
+        <v>-1.9999999999999574E-2</v>
+      </c>
+      <c r="E79" s="8">
+        <f t="shared" si="19"/>
+        <v>-0.14000000000000057</v>
       </c>
     </row>
   </sheetData>

</xml_diff>